<commit_message>
Adds some comments to BOM. Parts have been ordered
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Inverter/Rev04/BOM/BOM_UZ_D_Inverter_Variant_V1_Rev04.xlsx
+++ b/Project Outputs for UZ_D_Inverter/Rev04/BOM/BOM_UZ_D_Inverter_Variant_V1_Rev04.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_d_inverter\Project Outputs for UZ_D_Inverter\Rev04\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D447DA4-B828-476B-9512-1BA1A8EBA86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15BE2C61-EDE1-46B3-9EEA-E9677E938AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26916" yWindow="3804" windowWidth="23040" windowHeight="12120" xr2:uid="{F1393F58-CEFA-4786-B894-415FB3C9050D}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{F1393F58-CEFA-4786-B894-415FB3C9050D}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UZ_D_Inverter_Variant_V1_Re" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="197">
   <si>
     <t>Comment</t>
   </si>
@@ -600,6 +600,36 @@
   </si>
   <si>
     <t>SOT95P280X145-5N</t>
+  </si>
+  <si>
+    <t>BAT165E6327</t>
+  </si>
+  <si>
+    <t>C17913 </t>
+  </si>
+  <si>
+    <t>C151511</t>
+  </si>
+  <si>
+    <t>C318130</t>
+  </si>
+  <si>
+    <t>C16840</t>
+  </si>
+  <si>
+    <t>C17598</t>
+  </si>
+  <si>
+    <t>C2871658</t>
+  </si>
+  <si>
+    <t>replaced with:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08051C103J4Z2A </t>
+  </si>
+  <si>
+    <t>GlobalSourcing</t>
   </si>
 </sst>
 </file>
@@ -615,7 +645,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -628,8 +658,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -652,16 +700,44 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -996,788 +1072,817 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{639EC922-24AC-4BCD-BD2D-8588A8D15E21}">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
-    <col min="2" max="2" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="87.44140625" customWidth="1"/>
     <col min="3" max="3" width="23.88671875" customWidth="1"/>
-    <col min="4" max="5" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" customWidth="1"/>
+    <col min="5" max="5" width="57.33203125" customWidth="1"/>
+    <col min="6" max="6" width="19.77734375" customWidth="1"/>
+    <col min="7" max="7" width="17.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="F1" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="F3" s="8"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="F6" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="4" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="F13" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="4" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="4" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="4" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="4" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="4" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="4" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="4" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="4" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
+      <c r="F28" s="6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" s="4" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" s="4" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="4" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
+      <c r="F32" s="6" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="4" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E34" s="4" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
+      <c r="F34" s="6" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D35" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" s="4" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D36" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="4" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D37" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D38" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E38" s="4" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="D39" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="E39" s="4" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="D40" s="1"/>
-      <c r="E40" s="2" t="s">
+      <c r="D40" s="10"/>
+      <c r="E40" s="9" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="D41" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="4" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C42" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="D42" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E42" s="9" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C43" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="D43" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" s="9" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" s="2" t="s">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="D44" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="E44" s="4" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="C45" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="D45" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" s="4" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C46" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="D46" s="1"/>
-      <c r="E46" s="2" t="s">
+      <c r="D46" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="E46" s="4" t="s">
         <v>184</v>
       </c>
     </row>

</xml_diff>